<commit_message>
Reorganise chapters: extract Roadmap, move scenario analysis
- Split GTM Adoption Strategy out of chap 10 into new chap_roadmap.tex
- Reorder includes: competitive -> roadmap -> regulatory -> business -> gtm
- Move Scenario Analysis from risk chapter to financial chapter as final section
- Update intros/conclusions and internal cross-references accordingly
</commit_message>
<xml_diff>
--- a/financial_model.xlsx
+++ b/financial_model.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="487">
   <si>
     <t xml:space="preserve">mTBI Screening Tool — Financial Model — Assumptions</t>
   </si>
@@ -210,7 +210,7 @@
     <t xml:space="preserve">£/sub/yr</t>
   </si>
   <si>
-    <t xml:space="preserve"> = $B$27 (single-tier per-headset pricing)</t>
+    <t xml:space="preserve"> = $B$27 × ARPU scenario multiplier</t>
   </si>
   <si>
     <t xml:space="preserve">Subscription attach (per institutional headset)</t>
@@ -612,7 +612,7 @@
     <t xml:space="preserve">Equity injections</t>
   </si>
   <si>
-    <t xml:space="preserve">Mechanical plug — sized to keep closing cash ≥ buffer at all times</t>
+    <t xml:space="preserve">Pre-seed Y1 / Seed Y3 / Seed-2 Y5 per ch.12 §12.2 (total £4.2M, 12% buffer over £3.75M trough)</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum cash buffer</t>
@@ -837,7 +837,7 @@
     <t xml:space="preserve">Hardware revenue</t>
   </si>
   <si>
-    <t xml:space="preserve">delay-shifted new units × adoption scenario × ASP × (1 − returns allowance)</t>
+    <t xml:space="preserve">delay-shifted new units × adoption × ASP × ASP scenario × (1 − returns allowance)</t>
   </si>
   <si>
     <t xml:space="preserve">Subscription revenue</t>
@@ -1296,7 +1296,7 @@
     <t xml:space="preserve">1. SCENARIO SELECTOR</t>
   </si>
   <si>
-    <t xml:space="preserve">Active scenario  (1 = Base, 2 = Downside, 3 = Upside, 4 = Reg Delay)</t>
+    <t xml:space="preserve">Active scenario  (1=Base, 2=Downside, 3=Upside, 4=RegDelay, 5=Best, 6=Worst)</t>
   </si>
   <si>
     <t xml:space="preserve">Active scenario name</t>
@@ -1320,49 +1320,64 @@
     <t xml:space="preserve">Reg Delay</t>
   </si>
   <si>
+    <t xml:space="preserve">Best</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worst</t>
+  </si>
+  <si>
     <t xml:space="preserve">Interpretation</t>
   </si>
   <si>
     <t xml:space="preserve">Adoption ramp multiplier</t>
   </si>
   <si>
-    <t xml:space="preserve">Slow ramp (0.5×) vs fast ramp (1.3×); delay shifts curve separately</t>
+    <t xml:space="preserve">ch.13 Best/Worst: ±20% adoption around base</t>
   </si>
   <si>
     <t xml:space="preserve">BOM unit cost multiplier</t>
   </si>
   <si>
-    <t xml:space="preserve">Component price spike vs improved sourcing</t>
+    <t xml:space="preserve">ch.13 Worst: cost-down slips, +20-30% (use 25%); Best: -10%</t>
   </si>
   <si>
     <t xml:space="preserve">Subscription churn multiplier</t>
   </si>
   <si>
-    <t xml:space="preserve">15% churn vs 7% churn</t>
+    <t xml:space="preserve">ch.13: Best 8% (×0.8), Worst 15% (×1.5) from 10% base</t>
   </si>
   <si>
     <t xml:space="preserve">Headcount / payroll multiplier</t>
   </si>
   <si>
-    <t xml:space="preserve">Reg Delay: team runs longer, +5% cumulative payroll</t>
+    <t xml:space="preserve">ch.13 Worst: burn +10% via payroll lever (dominant cost)</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing spend multiplier</t>
   </si>
   <si>
-    <t xml:space="preserve">Less efficient acquisition vs better channels</t>
+    <t xml:space="preserve">ch.13 Best/Worst hold marketing flat; effect routed via payroll</t>
   </si>
   <si>
     <t xml:space="preserve">Regulatory &amp; clinical multiplier</t>
   </si>
   <si>
-    <t xml:space="preserve">Reg Delay: more NB fees, extra clinical data (+40%)</t>
+    <t xml:space="preserve">Worst: extra NB / clinical cost from delay (+20%)</t>
   </si>
   <si>
     <t xml:space="preserve">Regulatory delay  (years shifted)</t>
   </si>
   <si>
-    <t xml:space="preserve">Shifts commercial adoption curve right by N years</t>
+    <t xml:space="preserve">ch.13 Worst: 12-month MDR slip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware ASP multiplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ch.13: Best +10%, Worst -12.5% (mid of -10/-15%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subscription ARPU multiplier</t>
   </si>
   <si>
     <t xml:space="preserve">3. ACTIVE MULTIPLIERS  (live values used by Assumptions and P&amp;L)</t>
@@ -1387,6 +1402,12 @@
   </si>
   <si>
     <t xml:space="preserve">Regulatory delay  (years, active)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware ASP multiplier (active)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subscription ARPU multiplier (active)</t>
   </si>
   <si>
     <t xml:space="preserve">4. ACTIVE SCENARIO HEADLINE OUTPUTS  (live, recomputes when selector changes)</t>
@@ -2398,31 +2419,31 @@
         <v>29</v>
       </c>
       <c r="C17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(C5 - Scenarios!$B$24, MIN(C5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(C17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(C5 - Scenarios!$B$26, MIN(C5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(C17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>0</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(D5 - Scenarios!$B$24, MIN(D5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(D17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(D5 - Scenarios!$B$26, MIN(D5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(D17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>0</v>
       </c>
       <c r="E17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(E5 - Scenarios!$B$24, MIN(E5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(E17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(E5 - Scenarios!$B$26, MIN(E5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(E17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>90</v>
       </c>
       <c r="F17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(F5 - Scenarios!$B$24, MIN(F5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(F17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(F5 - Scenarios!$B$26, MIN(F5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(F17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>351</v>
       </c>
       <c r="G17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(G5 - Scenarios!$B$24, MIN(G5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(G17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(G5 - Scenarios!$B$26, MIN(G5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(G17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>765.9</v>
       </c>
       <c r="H17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(H5 - Scenarios!$B$24, MIN(H5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(H17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(H5 - Scenarios!$B$26, MIN(H5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(H17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>1889.31</v>
       </c>
       <c r="I17" s="9" t="n">
-        <f aca="true">INDEX($C$28:$K$28, 1, MAX(I5 - Scenarios!$B$24, MIN(I5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 + OFFSET(I17, 0, -1) * (1 - $B$16 * Scenarios!$B$20)</f>
+        <f aca="true">INDEX($C$28:$K$28, 1, MAX(I5 - Scenarios!$B$26, MIN(I5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 + OFFSET(I17, 0, -1) * (1 - $B$16 * Scenarios!$B$22)</f>
         <v>3950.379</v>
       </c>
       <c r="L17" s="6" t="s">
@@ -2476,31 +2497,31 @@
         <v>34</v>
       </c>
       <c r="C19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(C5 - Scenarios!$B$24, MIN(C5, 3))) * Scenarios!$B$18 + OFFSET(C19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(C5 - Scenarios!$B$26, MIN(C5, 3))) * Scenarios!$B$20 + OFFSET(C19, 0, -1)</f>
         <v>0</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(D5 - Scenarios!$B$24, MIN(D5, 3))) * Scenarios!$B$18 + OFFSET(D19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(D5 - Scenarios!$B$26, MIN(D5, 3))) * Scenarios!$B$20 + OFFSET(D19, 0, -1)</f>
         <v>0</v>
       </c>
       <c r="E19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(E5 - Scenarios!$B$24, MIN(E5, 3))) * Scenarios!$B$18 + OFFSET(E19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(E5 - Scenarios!$B$26, MIN(E5, 3))) * Scenarios!$B$20 + OFFSET(E19, 0, -1)</f>
         <v>90</v>
       </c>
       <c r="F19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(F5 - Scenarios!$B$24, MIN(F5, 3))) * Scenarios!$B$18 + OFFSET(F19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(F5 - Scenarios!$B$26, MIN(F5, 3))) * Scenarios!$B$20 + OFFSET(F19, 0, -1)</f>
         <v>360</v>
       </c>
       <c r="G19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(G5 - Scenarios!$B$24, MIN(G5, 3))) * Scenarios!$B$18 + OFFSET(G19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(G5 - Scenarios!$B$26, MIN(G5, 3))) * Scenarios!$B$20 + OFFSET(G19, 0, -1)</f>
         <v>1851</v>
       </c>
       <c r="H19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(H5 - Scenarios!$B$24, MIN(H5, 3))) * Scenarios!$B$18 + OFFSET(H19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(H5 - Scenarios!$B$26, MIN(H5, 3))) * Scenarios!$B$20 + OFFSET(H19, 0, -1)</f>
         <v>5005</v>
       </c>
       <c r="I19" s="9" t="n">
-        <f aca="true">INDEX($C$15:$K$15, 1, MAX(I5 - Scenarios!$B$24, MIN(I5, 3))) * Scenarios!$B$18 + OFFSET(I19, 0, -1)</f>
+        <f aca="true">INDEX($C$15:$K$15, 1, MAX(I5 - Scenarios!$B$26, MIN(I5, 3))) * Scenarios!$B$20 + OFFSET(I19, 0, -1)</f>
         <v>12580</v>
       </c>
       <c r="L19" s="6" t="s">
@@ -2749,31 +2770,31 @@
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="D32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="E32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="F32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="G32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="H32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="I32" s="16" t="n">
-        <f aca="false">$B$27</f>
+        <f aca="false">$B$27 * Scenarios!$B$28</f>
         <v>600</v>
       </c>
       <c r="J32" s="15"/>
@@ -3008,31 +3029,31 @@
         <v>89</v>
       </c>
       <c r="C49" s="19" t="n">
-        <f aca="false">CHOOSE(C7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(C7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>340</v>
       </c>
       <c r="D49" s="19" t="n">
-        <f aca="false">CHOOSE(D7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(D7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>340</v>
       </c>
       <c r="E49" s="19" t="n">
-        <f aca="false">CHOOSE(E7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(E7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>285</v>
       </c>
       <c r="F49" s="19" t="n">
-        <f aca="false">CHOOSE(F7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(F7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>285</v>
       </c>
       <c r="G49" s="19" t="n">
-        <f aca="false">CHOOSE(G7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(G7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>174</v>
       </c>
       <c r="H49" s="19" t="n">
-        <f aca="false">CHOOSE(H7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(H7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>174</v>
       </c>
       <c r="I49" s="19" t="n">
-        <f aca="false">CHOOSE(I7, $B$46, $B$47, $B$48) * Scenarios!$B$19</f>
+        <f aca="false">CHOOSE(I7, $B$46, $B$47, $B$48) * Scenarios!$B$21</f>
         <v>174</v>
       </c>
       <c r="L49" s="6" t="s">
@@ -3454,31 +3475,31 @@
         <v>118</v>
       </c>
       <c r="C66" s="19" t="n">
-        <f aca="false">(C63 + C64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(C63 + C64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>220150</v>
       </c>
       <c r="D66" s="19" t="n">
-        <f aca="false">(D63 + D64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(D63 + D64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>282625</v>
       </c>
       <c r="E66" s="19" t="n">
-        <f aca="false">(E63 + E64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(E63 + E64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>503370</v>
       </c>
       <c r="F66" s="19" t="n">
-        <f aca="false">(F63 + F64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(F63 + F64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>737205</v>
       </c>
       <c r="G66" s="19" t="n">
-        <f aca="false">(G63 + G64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(G63 + G64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>917490</v>
       </c>
       <c r="H66" s="19" t="n">
-        <f aca="false">(H63 + H64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(H63 + H64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>1001980</v>
       </c>
       <c r="I66" s="19" t="n">
-        <f aca="false">(I63 + I64) * (1 + $B$65) * Scenarios!$B$21</f>
+        <f aca="false">(I63 + I64) * (1 + $B$65) * Scenarios!$B$23</f>
         <v>1086470</v>
       </c>
       <c r="L66" s="6" t="s">
@@ -3507,31 +3528,31 @@
         <v>123</v>
       </c>
       <c r="C68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(C5 - Scenarios!$B$24, MIN(C5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * C32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(C5 - Scenarios!$B$26, MIN(C5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * C32 * $B$67</f>
         <v>0</v>
       </c>
       <c r="D68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(D5 - Scenarios!$B$24, MIN(D5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * D32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(D5 - Scenarios!$B$26, MIN(D5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * D32 * $B$67</f>
         <v>0</v>
       </c>
       <c r="E68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(E5 - Scenarios!$B$24, MIN(E5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * E32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(E5 - Scenarios!$B$26, MIN(E5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * E32 * $B$67</f>
         <v>8100</v>
       </c>
       <c r="F68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(F5 - Scenarios!$B$24, MIN(F5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * F32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(F5 - Scenarios!$B$26, MIN(F5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * F32 * $B$67</f>
         <v>24300</v>
       </c>
       <c r="G68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(G5 - Scenarios!$B$24, MIN(G5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * G32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(G5 - Scenarios!$B$26, MIN(G5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * G32 * $B$67</f>
         <v>40500</v>
       </c>
       <c r="H68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(H5 - Scenarios!$B$24, MIN(H5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * H32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(H5 - Scenarios!$B$26, MIN(H5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * H32 * $B$67</f>
         <v>108000</v>
       </c>
       <c r="I68" s="19" t="n">
-        <f aca="false">INDEX($C$28:$K$28, 1, MAX(I5 - Scenarios!$B$24, MIN(I5, 3))) * $B$26 * Scenarios!$B$18 * $B$33 * I32 * $B$67</f>
+        <f aca="false">INDEX($C$28:$K$28, 1, MAX(I5 - Scenarios!$B$26, MIN(I5, 3))) * $B$26 * Scenarios!$B$20 * $B$33 * I32 * $B$67</f>
         <v>202500</v>
       </c>
       <c r="L68" s="6" t="s">
@@ -4591,19 +4612,19 @@
         <v>194</v>
       </c>
       <c r="C126" s="11" t="n">
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="D126" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E126" s="11" t="n">
-        <v>1500000</v>
+        <v>1750000</v>
       </c>
       <c r="F126" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G126" s="11" t="n">
-        <v>1500000</v>
+        <v>1450000</v>
       </c>
       <c r="H126" s="11" t="n">
         <v>0</v>
@@ -6814,31 +6835,31 @@
         <v>269</v>
       </c>
       <c r="C9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(C5 - Scenarios!$B$24, MIN(C5, 3))) * Scenarios!$B$18 * Assumptions!C22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(C5 - Scenarios!$B$26, MIN(C5, 3))) * Scenarios!$B$20 * Assumptions!C22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>0</v>
       </c>
       <c r="D9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(D5 - Scenarios!$B$24, MIN(D5, 3))) * Scenarios!$B$18 * Assumptions!D22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(D5 - Scenarios!$B$26, MIN(D5, 3))) * Scenarios!$B$20 * Assumptions!D22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>0</v>
       </c>
       <c r="E9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(E5 - Scenarios!$B$24, MIN(E5, 3))) * Scenarios!$B$18 * Assumptions!E22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(E5 - Scenarios!$B$26, MIN(E5, 3))) * Scenarios!$B$20 * Assumptions!E22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>26460</v>
       </c>
       <c r="F9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(F5 - Scenarios!$B$24, MIN(F5, 3))) * Scenarios!$B$18 * Assumptions!F22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(F5 - Scenarios!$B$26, MIN(F5, 3))) * Scenarios!$B$20 * Assumptions!F22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>79380</v>
       </c>
       <c r="G9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(G5 - Scenarios!$B$24, MIN(G5, 3))) * Scenarios!$B$18 * Assumptions!G22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(G5 - Scenarios!$B$26, MIN(G5, 3))) * Scenarios!$B$20 * Assumptions!G22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>438354</v>
       </c>
       <c r="H9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(H5 - Scenarios!$B$24, MIN(H5, 3))) * Scenarios!$B$18 * Assumptions!H22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(H5 - Scenarios!$B$26, MIN(H5, 3))) * Scenarios!$B$20 * Assumptions!H22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>927276</v>
       </c>
       <c r="I9" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(I5 - Scenarios!$B$24, MIN(I5, 3))) * Scenarios!$B$18 * Assumptions!I22 * (1 - Assumptions!$B$23)</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(I5 - Scenarios!$B$26, MIN(I5, 3))) * Scenarios!$B$20 * Assumptions!I22 * Scenarios!$B$27 * (1 - Assumptions!$B$23)</f>
         <v>2227050</v>
       </c>
       <c r="L9" s="6" t="s">
@@ -6970,31 +6991,31 @@
         <v>277</v>
       </c>
       <c r="C13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(C5 - Scenarios!$B$24, MIN(C5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(C5 - Scenarios!$B$26, MIN(C5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="D13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(D5 - Scenarios!$B$24, MIN(D5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(D5 - Scenarios!$B$26, MIN(D5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="E13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(E5 - Scenarios!$B$24, MIN(E5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(E5 - Scenarios!$B$26, MIN(E5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="F13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(F5 - Scenarios!$B$24, MIN(F5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(F5 - Scenarios!$B$26, MIN(F5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="G13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(G5 - Scenarios!$B$24, MIN(G5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(G5 - Scenarios!$B$26, MIN(G5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="H13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(H5 - Scenarios!$B$24, MIN(H5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(H5 - Scenarios!$B$26, MIN(H5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="I13" s="19" t="n">
-        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(I5 - Scenarios!$B$24, MIN(I5, 3))) * Scenarios!$B$18 * Assumptions!$B$42 * Assumptions!$B$43</f>
+        <f aca="false">Assumptions!$B$41 * INDEX(Assumptions!$C$15:$K$15, 1, MAX(I5 - Scenarios!$B$26, MIN(I5, 3))) * Scenarios!$B$20 * Assumptions!$B$42 * Assumptions!$B$43</f>
         <v>0</v>
       </c>
       <c r="L13" s="6" t="s">
@@ -7066,31 +7087,31 @@
         <v>281</v>
       </c>
       <c r="C17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(C5 - Scenarios!$B$24, MIN(C5, 3))) * Scenarios!$B$18 * Assumptions!C49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(C5 - Scenarios!$B$26, MIN(C5, 3))) * Scenarios!$B$20 * Assumptions!C49</f>
         <v>0</v>
       </c>
       <c r="D17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(D5 - Scenarios!$B$24, MIN(D5, 3))) * Scenarios!$B$18 * Assumptions!D49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(D5 - Scenarios!$B$26, MIN(D5, 3))) * Scenarios!$B$20 * Assumptions!D49</f>
         <v>0</v>
       </c>
       <c r="E17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(E5 - Scenarios!$B$24, MIN(E5, 3))) * Scenarios!$B$18 * Assumptions!E49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(E5 - Scenarios!$B$26, MIN(E5, 3))) * Scenarios!$B$20 * Assumptions!E49</f>
         <v>25650</v>
       </c>
       <c r="F17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(F5 - Scenarios!$B$24, MIN(F5, 3))) * Scenarios!$B$18 * Assumptions!F49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(F5 - Scenarios!$B$26, MIN(F5, 3))) * Scenarios!$B$20 * Assumptions!F49</f>
         <v>76950</v>
       </c>
       <c r="G17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(G5 - Scenarios!$B$24, MIN(G5, 3))) * Scenarios!$B$18 * Assumptions!G49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(G5 - Scenarios!$B$26, MIN(G5, 3))) * Scenarios!$B$20 * Assumptions!G49</f>
         <v>259434</v>
       </c>
       <c r="H17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(H5 - Scenarios!$B$24, MIN(H5, 3))) * Scenarios!$B$18 * Assumptions!H49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(H5 - Scenarios!$B$26, MIN(H5, 3))) * Scenarios!$B$20 * Assumptions!H49</f>
         <v>548796</v>
       </c>
       <c r="I17" s="19" t="n">
-        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(I5 - Scenarios!$B$24, MIN(I5, 3))) * Scenarios!$B$18 * Assumptions!I49</f>
+        <f aca="false">INDEX(Assumptions!$C$15:$K$15, 1, MAX(I5 - Scenarios!$B$26, MIN(I5, 3))) * Scenarios!$B$20 * Assumptions!I49</f>
         <v>1318050</v>
       </c>
       <c r="L17" s="6" t="s">
@@ -7553,31 +7574,31 @@
         <v>297</v>
       </c>
       <c r="C34" s="19" t="n">
-        <f aca="false">Assumptions!C86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!C86 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="D34" s="19" t="n">
-        <f aca="false">Assumptions!D86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!D86 * Scenarios!$B$25</f>
         <v>130000</v>
       </c>
       <c r="E34" s="19" t="n">
-        <f aca="false">Assumptions!E86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!E86 * Scenarios!$B$25</f>
         <v>140000</v>
       </c>
       <c r="F34" s="19" t="n">
-        <f aca="false">Assumptions!F86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!F86 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="G34" s="19" t="n">
-        <f aca="false">Assumptions!G86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!G86 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="H34" s="19" t="n">
-        <f aca="false">Assumptions!H86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!H86 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="I34" s="19" t="n">
-        <f aca="false">Assumptions!I86 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!I86 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="L34" s="6" t="s">
@@ -7592,31 +7613,31 @@
         <v>299</v>
       </c>
       <c r="C35" s="19" t="n">
-        <f aca="false">Assumptions!C87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!C87 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="D35" s="19" t="n">
-        <f aca="false">Assumptions!D87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!D87 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="E35" s="19" t="n">
-        <f aca="false">Assumptions!E87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!E87 * Scenarios!$B$25</f>
         <v>0</v>
       </c>
       <c r="F35" s="19" t="n">
-        <f aca="false">Assumptions!F87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!F87 * Scenarios!$B$25</f>
         <v>55000</v>
       </c>
       <c r="G35" s="19" t="n">
-        <f aca="false">Assumptions!G87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!G87 * Scenarios!$B$25</f>
         <v>55000</v>
       </c>
       <c r="H35" s="19" t="n">
-        <f aca="false">Assumptions!H87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!H87 * Scenarios!$B$25</f>
         <v>60000</v>
       </c>
       <c r="I35" s="19" t="n">
-        <f aca="false">Assumptions!I87 * Scenarios!$B$23</f>
+        <f aca="false">Assumptions!I87 * Scenarios!$B$25</f>
         <v>65000</v>
       </c>
       <c r="L35" s="6" t="s">
@@ -7796,31 +7817,31 @@
         <v>306</v>
       </c>
       <c r="C42" s="19" t="n">
-        <f aca="false">Assumptions!C73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!C73 * Scenarios!$B$24</f>
         <v>5000</v>
       </c>
       <c r="D42" s="19" t="n">
-        <f aca="false">Assumptions!D73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!D73 * Scenarios!$B$24</f>
         <v>10000</v>
       </c>
       <c r="E42" s="19" t="n">
-        <f aca="false">Assumptions!E73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!E73 * Scenarios!$B$24</f>
         <v>25000</v>
       </c>
       <c r="F42" s="19" t="n">
-        <f aca="false">Assumptions!F73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!F73 * Scenarios!$B$24</f>
         <v>50000</v>
       </c>
       <c r="G42" s="19" t="n">
-        <f aca="false">Assumptions!G73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!G73 * Scenarios!$B$24</f>
         <v>150000</v>
       </c>
       <c r="H42" s="19" t="n">
-        <f aca="false">Assumptions!H73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!H73 * Scenarios!$B$24</f>
         <v>300000</v>
       </c>
       <c r="I42" s="19" t="n">
-        <f aca="false">Assumptions!I73 * Scenarios!$B$22</f>
+        <f aca="false">Assumptions!I73 * Scenarios!$B$24</f>
         <v>500000</v>
       </c>
       <c r="L42" s="6" t="s">
@@ -8417,27 +8438,27 @@
       </c>
       <c r="D64" s="19" t="n">
         <f aca="false">'Cash flow'!D38 * Assumptions!$B$124</f>
-        <v>19534.7838928958</v>
+        <v>22534.7838928958</v>
       </c>
       <c r="E64" s="19" t="n">
         <f aca="false">'Cash flow'!E38 * Assumptions!$B$124</f>
-        <v>6424.10175560512</v>
+        <v>9514.10175560512</v>
       </c>
       <c r="F64" s="19" t="n">
         <f aca="false">'Cash flow'!F38 * Assumptions!$B$124</f>
-        <v>29354.3875753966</v>
+        <v>40037.0875753966</v>
       </c>
       <c r="G64" s="19" t="n">
         <f aca="false">'Cash flow'!G38 * Assumptions!$B$124</f>
-        <v>3291.75993690503</v>
+        <v>14294.940936905</v>
       </c>
       <c r="H64" s="19" t="n">
         <f aca="false">'Cash flow'!H38 * Assumptions!$B$124</f>
-        <v>21331.6158884368</v>
+        <v>31164.8923184368</v>
       </c>
       <c r="I64" s="19" t="n">
         <f aca="false">'Cash flow'!I38 * Assumptions!$B$124</f>
-        <v>4614.45813906255</v>
+        <v>14742.7328619626</v>
       </c>
       <c r="L64" s="6" t="s">
         <v>113</v>
@@ -8477,23 +8498,23 @@
       </c>
       <c r="E66" s="19" t="n">
         <f aca="true">OFFSET(E66, 7, -1)</f>
-        <v>766040.216107104</v>
+        <v>763040.216107104</v>
       </c>
       <c r="F66" s="19" t="n">
         <f aca="true">OFFSET(F66, 7, -1)</f>
-        <v>1561826.1143515</v>
+        <v>1555736.1143515</v>
       </c>
       <c r="G66" s="19" t="n">
         <f aca="true">OFFSET(G66, 7, -1)</f>
-        <v>2501591.7267761</v>
+        <v>2484819.0267761</v>
       </c>
       <c r="H66" s="19" t="n">
         <f aca="true">OFFSET(H66, 7, -1)</f>
-        <v>3484060.4668392</v>
+        <v>3456284.5858392</v>
       </c>
       <c r="I66" s="19" t="n">
         <f aca="true">OFFSET(I66, 7, -1)</f>
-        <v>4227750.30095076</v>
+        <v>4190141.14352076</v>
       </c>
       <c r="L66" s="6" t="s">
         <v>113</v>
@@ -8532,7 +8553,7 @@
       </c>
       <c r="I67" s="19" t="n">
         <f aca="false">MIN(I66, MAX(0, I63 + I64))</f>
-        <v>135222.295996206</v>
+        <v>145350.570719106</v>
       </c>
       <c r="L67" s="6" t="s">
         <v>113</v>
@@ -8747,27 +8768,27 @@
       </c>
       <c r="D73" s="19" t="n">
         <f aca="false">D66 + MAX(0, -(D63 + D64)) - D67</f>
-        <v>766040.216107104</v>
+        <v>763040.216107104</v>
       </c>
       <c r="E73" s="19" t="n">
         <f aca="false">E66 + MAX(0, -(E63 + E64)) - E67</f>
-        <v>1561826.1143515</v>
+        <v>1555736.1143515</v>
       </c>
       <c r="F73" s="19" t="n">
         <f aca="false">F66 + MAX(0, -(F63 + F64)) - F67</f>
-        <v>2501591.7267761</v>
+        <v>2484819.0267761</v>
       </c>
       <c r="G73" s="19" t="n">
         <f aca="false">G66 + MAX(0, -(G63 + G64)) - G67</f>
-        <v>3484060.4668392</v>
+        <v>3456284.5858392</v>
       </c>
       <c r="H73" s="19" t="n">
         <f aca="false">H66 + MAX(0, -(H63 + H64)) - H67</f>
-        <v>4227750.30095076</v>
+        <v>4190141.14352076</v>
       </c>
       <c r="I73" s="19" t="n">
         <f aca="false">I66 + MAX(0, -(I63 + I64)) - I67</f>
-        <v>4092528.00495456</v>
+        <v>4044790.57280165</v>
       </c>
       <c r="L73" s="6" t="s">
         <v>113</v>
@@ -8787,27 +8808,27 @@
       </c>
       <c r="D75" s="16" t="n">
         <f aca="false">D63 + D64 - D72</f>
-        <v>-455591.231060375</v>
+        <v>-452591.231060375</v>
       </c>
       <c r="E75" s="16" t="n">
         <f aca="false">E63 + E64 - E72</f>
-        <v>-740488.098244395</v>
+        <v>-737398.098244395</v>
       </c>
       <c r="F75" s="16" t="n">
         <f aca="false">F63 + F64 - F72</f>
-        <v>-886376.172424604</v>
+        <v>-875693.472424604</v>
       </c>
       <c r="G75" s="16" t="n">
         <f aca="false">G63 + G64 - G72</f>
-        <v>-918897.660063095</v>
+        <v>-907894.479063095</v>
       </c>
       <c r="H75" s="16" t="n">
         <f aca="false">H63 + H64 - H72</f>
-        <v>-672814.534111563</v>
+        <v>-662981.257681563</v>
       </c>
       <c r="I75" s="16" t="n">
         <f aca="false">I63 + I64 - I72</f>
-        <v>213401.815996206</v>
+        <v>223530.090719106</v>
       </c>
       <c r="J75" s="15"/>
       <c r="K75" s="15"/>
@@ -8830,23 +8851,23 @@
       </c>
       <c r="E76" s="28" t="n">
         <f aca="false">IFERROR(E75/E14, 0)</f>
-        <v>-13.8512551111933</v>
+        <v>-13.7934548867264</v>
       </c>
       <c r="F76" s="28" t="n">
         <f aca="false">IFERROR(F75/F14, 0)</f>
-        <v>-4.18734019474964</v>
+        <v>-4.13687392490837</v>
       </c>
       <c r="G76" s="28" t="n">
         <f aca="false">IFERROR(G75/G14, 0)</f>
-        <v>-1.18809043947834</v>
+        <v>-1.17386385612949</v>
       </c>
       <c r="H76" s="28" t="n">
         <f aca="false">IFERROR(H75/H14, 0)</f>
-        <v>-0.390300100016047</v>
+        <v>-0.384595810676962</v>
       </c>
       <c r="I76" s="28" t="n">
         <f aca="false">IFERROR(I75/I14, 0)</f>
-        <v>0.0536326057522078</v>
+        <v>0.0561780656520102</v>
       </c>
       <c r="L76" s="6" t="s">
         <v>75</v>
@@ -9592,27 +9613,27 @@
       </c>
       <c r="D25" s="27" t="n">
         <f aca="false">'P&amp;L'!D64</f>
-        <v>19534.7838928958</v>
+        <v>22534.7838928958</v>
       </c>
       <c r="E25" s="27" t="n">
         <f aca="false">'P&amp;L'!E64</f>
-        <v>6424.10175560512</v>
+        <v>9514.10175560512</v>
       </c>
       <c r="F25" s="27" t="n">
         <f aca="false">'P&amp;L'!F64</f>
-        <v>29354.3875753966</v>
+        <v>40037.0875753966</v>
       </c>
       <c r="G25" s="27" t="n">
         <f aca="false">'P&amp;L'!G64</f>
-        <v>3291.75993690503</v>
+        <v>14294.940936905</v>
       </c>
       <c r="H25" s="27" t="n">
         <f aca="false">'P&amp;L'!H64</f>
-        <v>21331.6158884368</v>
+        <v>31164.8923184368</v>
       </c>
       <c r="I25" s="27" t="n">
         <f aca="false">'P&amp;L'!I64</f>
-        <v>4614.45813906255</v>
+        <v>14742.7328619626</v>
       </c>
       <c r="L25" s="6" t="s">
         <v>113</v>
@@ -9632,27 +9653,27 @@
       </c>
       <c r="D26" s="16" t="n">
         <f aca="false">D13 + D24 + D25</f>
-        <v>-431022.73790969</v>
+        <v>-428022.73790969</v>
       </c>
       <c r="E26" s="16" t="n">
         <f aca="false">E13 + E24 + E25</f>
-        <v>-720657.139340285</v>
+        <v>-717567.139340285</v>
       </c>
       <c r="F26" s="16" t="n">
         <f aca="false">F13 + F24 + F25</f>
-        <v>-848754.254616384</v>
+        <v>-838071.554616384</v>
       </c>
       <c r="G26" s="16" t="n">
         <f aca="false">G13 + G24 + G25</f>
-        <v>-868671.468282273</v>
+        <v>-857668.287282273</v>
       </c>
       <c r="H26" s="16" t="n">
         <f aca="false">H13 + H24 + H25</f>
-        <v>-545238.59164581</v>
+        <v>-535405.31521581</v>
       </c>
       <c r="I26" s="16" t="n">
         <f aca="false">I13 + I24 + I25</f>
-        <v>389378.267933584</v>
+        <v>399506.542656484</v>
       </c>
       <c r="J26" s="15"/>
       <c r="K26" s="15"/>
@@ -9780,7 +9801,7 @@
       </c>
       <c r="C33" s="27" t="n">
         <f aca="false">Assumptions!C126</f>
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="D33" s="27" t="n">
         <f aca="false">Assumptions!D126</f>
@@ -9788,7 +9809,7 @@
       </c>
       <c r="E33" s="27" t="n">
         <f aca="false">Assumptions!E126</f>
-        <v>1500000</v>
+        <v>1750000</v>
       </c>
       <c r="F33" s="27" t="n">
         <f aca="false">Assumptions!F126</f>
@@ -9796,7 +9817,7 @@
       </c>
       <c r="G33" s="27" t="n">
         <f aca="false">Assumptions!G126</f>
-        <v>1500000</v>
+        <v>1450000</v>
       </c>
       <c r="H33" s="27" t="n">
         <f aca="false">Assumptions!H126</f>
@@ -9820,7 +9841,7 @@
       <c r="B34" s="15"/>
       <c r="C34" s="16" t="n">
         <f aca="false">C33</f>
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="D34" s="16" t="n">
         <f aca="false">D33</f>
@@ -9828,7 +9849,7 @@
       </c>
       <c r="E34" s="16" t="n">
         <f aca="false">E33</f>
-        <v>1500000</v>
+        <v>1750000</v>
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">F33</f>
@@ -9836,7 +9857,7 @@
       </c>
       <c r="G34" s="16" t="n">
         <f aca="false">G33</f>
-        <v>1500000</v>
+        <v>1450000</v>
       </c>
       <c r="H34" s="16" t="n">
         <f aca="false">H33</f>
@@ -9876,31 +9897,31 @@
       </c>
       <c r="C37" s="19" t="n">
         <f aca="false">C26 + C30 + C34</f>
-        <v>651159.463096528</v>
+        <v>751159.463096528</v>
       </c>
       <c r="D37" s="19" t="n">
         <f aca="false">D26 + D30 + D34</f>
-        <v>-437022.73790969</v>
+        <v>-434022.73790969</v>
       </c>
       <c r="E37" s="19" t="n">
         <f aca="false">E26 + E30 + E34</f>
-        <v>764342.860659715</v>
+        <v>1017432.86065971</v>
       </c>
       <c r="F37" s="19" t="n">
         <f aca="false">F26 + F30 + F34</f>
-        <v>-868754.254616384</v>
+        <v>-858071.554616384</v>
       </c>
       <c r="G37" s="19" t="n">
         <f aca="false">G26 + G30 + G34</f>
-        <v>601328.531717727</v>
+        <v>562331.712717727</v>
       </c>
       <c r="H37" s="19" t="n">
         <f aca="false">H26 + H30 + H34</f>
-        <v>-557238.59164581</v>
+        <v>-547405.31521581</v>
       </c>
       <c r="I37" s="19" t="n">
         <f aca="false">I26 + I30 + I34</f>
-        <v>367378.267933584</v>
+        <v>377506.542656484</v>
       </c>
       <c r="L37" s="6" t="s">
         <v>113</v>
@@ -9916,27 +9937,27 @@
       </c>
       <c r="D38" s="19" t="n">
         <f aca="true">OFFSET(D38, 1, -1)</f>
-        <v>651159.463096528</v>
+        <v>751159.463096528</v>
       </c>
       <c r="E38" s="19" t="n">
         <f aca="true">OFFSET(E38, 1, -1)</f>
-        <v>214136.725186837</v>
+        <v>317136.725186837</v>
       </c>
       <c r="F38" s="19" t="n">
         <f aca="true">OFFSET(F38, 1, -1)</f>
-        <v>978479.585846552</v>
+        <v>1334569.58584655</v>
       </c>
       <c r="G38" s="19" t="n">
         <f aca="true">OFFSET(G38, 1, -1)</f>
-        <v>109725.331230168</v>
+        <v>476498.031230168</v>
       </c>
       <c r="H38" s="19" t="n">
         <f aca="true">OFFSET(H38, 1, -1)</f>
-        <v>711053.862947895</v>
+        <v>1038829.74394789</v>
       </c>
       <c r="I38" s="19" t="n">
         <f aca="true">OFFSET(I38, 1, -1)</f>
-        <v>153815.271302085</v>
+        <v>491424.428732085</v>
       </c>
       <c r="L38" s="6" t="s">
         <v>113</v>
@@ -9949,31 +9970,31 @@
       <c r="B39" s="15"/>
       <c r="C39" s="16" t="n">
         <f aca="false">C38 + C37</f>
-        <v>651159.463096528</v>
+        <v>751159.463096528</v>
       </c>
       <c r="D39" s="16" t="n">
         <f aca="false">D38 + D37</f>
-        <v>214136.725186837</v>
+        <v>317136.725186837</v>
       </c>
       <c r="E39" s="16" t="n">
         <f aca="false">E38 + E37</f>
-        <v>978479.585846552</v>
+        <v>1334569.58584655</v>
       </c>
       <c r="F39" s="16" t="n">
         <f aca="false">F38 + F37</f>
-        <v>109725.331230168</v>
+        <v>476498.031230168</v>
       </c>
       <c r="G39" s="16" t="n">
         <f aca="false">G38 + G37</f>
-        <v>711053.862947895</v>
+        <v>1038829.74394789</v>
       </c>
       <c r="H39" s="16" t="n">
         <f aca="false">H38 + H37</f>
-        <v>153815.271302085</v>
+        <v>491424.428732085</v>
       </c>
       <c r="I39" s="16" t="n">
         <f aca="false">I38 + I37</f>
-        <v>521193.539235669</v>
+        <v>868930.971388569</v>
       </c>
       <c r="J39" s="15"/>
       <c r="K39" s="15"/>
@@ -10064,27 +10085,27 @@
       </c>
       <c r="D42" s="19" t="n">
         <f aca="true">D26 + D30 + OFFSET(D42, 0, -1)</f>
-        <v>-685863.274813163</v>
+        <v>-682863.274813163</v>
       </c>
       <c r="E42" s="19" t="n">
         <f aca="true">E26 + E30 + OFFSET(E42, 0, -1)</f>
-        <v>-1421520.41415345</v>
+        <v>-1415430.41415345</v>
       </c>
       <c r="F42" s="19" t="n">
         <f aca="true">F26 + F30 + OFFSET(F42, 0, -1)</f>
-        <v>-2290274.66876983</v>
+        <v>-2273501.96876983</v>
       </c>
       <c r="G42" s="19" t="n">
         <f aca="true">G26 + G30 + OFFSET(G42, 0, -1)</f>
-        <v>-3188946.13705211</v>
+        <v>-3161170.25605211</v>
       </c>
       <c r="H42" s="19" t="n">
         <f aca="true">H26 + H30 + OFFSET(H42, 0, -1)</f>
-        <v>-3746184.72869792</v>
+        <v>-3708575.57126792</v>
       </c>
       <c r="I42" s="19" t="n">
         <f aca="true">I26 + I30 + OFFSET(I42, 0, -1)</f>
-        <v>-3378806.46076433</v>
+        <v>-3331069.02861143</v>
       </c>
       <c r="L42" s="6" t="s">
         <v>113</v>
@@ -10116,7 +10137,7 @@
       </c>
       <c r="B45" s="39" t="n">
         <f aca="false">MIN(C39:I39)</f>
-        <v>109725.331230168</v>
+        <v>317136.725186837</v>
       </c>
       <c r="C45" s="36"/>
       <c r="D45" s="36"/>
@@ -10140,7 +10161,7 @@
       </c>
       <c r="B46" s="41" t="str">
         <f aca="false">INDEX($C$4:$K$4, MATCH(MIN(C39:I39), C39:I39, 0))</f>
-        <v>Y4</v>
+        <v>Y2</v>
       </c>
       <c r="C46" s="36"/>
       <c r="D46" s="36"/>
@@ -10160,7 +10181,7 @@
       </c>
       <c r="B47" s="39" t="n">
         <f aca="false">MIN(C42:K42)</f>
-        <v>-3746184.72869792</v>
+        <v>-3708575.57126792</v>
       </c>
       <c r="C47" s="36"/>
       <c r="D47" s="36"/>
@@ -10204,7 +10225,7 @@
       </c>
       <c r="B49" s="39" t="n">
         <f aca="false">SUM(C33:K33)</f>
-        <v>3900000</v>
+        <v>4200000</v>
       </c>
       <c r="C49" s="36"/>
       <c r="D49" s="36"/>
@@ -10226,7 +10247,7 @@
       </c>
       <c r="B50" s="39" t="n">
         <f aca="false">SUM(C26:K26)</f>
-        <v>-3267306.46076433</v>
+        <v>-3219569.02861143</v>
       </c>
       <c r="C50" s="36"/>
       <c r="D50" s="36"/>
@@ -10495,31 +10516,31 @@
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">'Cash flow'!C39</f>
-        <v>651159.463096528</v>
+        <v>751159.463096528</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">'Cash flow'!D39</f>
-        <v>214136.725186837</v>
+        <v>317136.725186837</v>
       </c>
       <c r="E9" s="27" t="n">
         <f aca="false">'Cash flow'!E39</f>
-        <v>978479.585846552</v>
+        <v>1334569.58584655</v>
       </c>
       <c r="F9" s="27" t="n">
         <f aca="false">'Cash flow'!F39</f>
-        <v>109725.331230168</v>
+        <v>476498.031230168</v>
       </c>
       <c r="G9" s="27" t="n">
         <f aca="false">'Cash flow'!G39</f>
-        <v>711053.862947895</v>
+        <v>1038829.74394789</v>
       </c>
       <c r="H9" s="27" t="n">
         <f aca="false">'Cash flow'!H39</f>
-        <v>153815.271302085</v>
+        <v>491424.428732085</v>
       </c>
       <c r="I9" s="27" t="n">
         <f aca="false">'Cash flow'!I39</f>
-        <v>521193.539235669</v>
+        <v>868930.971388569</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>113</v>
@@ -10604,31 +10625,31 @@
       <c r="B12" s="15"/>
       <c r="C12" s="16" t="n">
         <f aca="false">SUM(C9:C11)</f>
-        <v>651159.463096528</v>
+        <v>751159.463096528</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">SUM(D9:D11)</f>
-        <v>214136.725186837</v>
+        <v>317136.725186837</v>
       </c>
       <c r="E12" s="16" t="n">
         <f aca="false">SUM(E9:E11)</f>
-        <v>991173.284476689</v>
+        <v>1347263.28447669</v>
       </c>
       <c r="F12" s="16" t="n">
         <f aca="false">SUM(F9:F11)</f>
-        <v>155712.249038387</v>
+        <v>522484.949038387</v>
       </c>
       <c r="G12" s="16" t="n">
         <f aca="false">SUM(G9:G11)</f>
-        <v>870043.362947895</v>
+        <v>1197819.24394789</v>
       </c>
       <c r="H12" s="16" t="n">
         <f aca="false">SUM(H9:H11)</f>
-        <v>503661.267877427</v>
+        <v>841270.425307428</v>
       </c>
       <c r="I12" s="16" t="n">
         <f aca="false">SUM(I9:I11)</f>
-        <v>1336579.16081101</v>
+        <v>1684316.59296391</v>
       </c>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
@@ -10756,31 +10777,31 @@
       <c r="B18" s="15"/>
       <c r="C18" s="16" t="n">
         <f aca="false">C12 + C16</f>
-        <v>656359.463096528</v>
+        <v>756359.463096528</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">D12 + D16</f>
-        <v>222836.725186837</v>
+        <v>325836.725186837</v>
       </c>
       <c r="E18" s="16" t="n">
         <f aca="false">E12 + E16</f>
-        <v>1009373.28447669</v>
+        <v>1365463.28447669</v>
       </c>
       <c r="F18" s="16" t="n">
         <f aca="false">F12 + F16</f>
-        <v>184412.249038387</v>
+        <v>551184.949038387</v>
       </c>
       <c r="G18" s="16" t="n">
         <f aca="false">G12 + G16</f>
-        <v>913243.362947895</v>
+        <v>1241019.24394789</v>
       </c>
       <c r="H18" s="16" t="n">
         <f aca="false">H12 + H16</f>
-        <v>542261.267877427</v>
+        <v>879870.425307428</v>
       </c>
       <c r="I18" s="16" t="n">
         <f aca="false">I12 + I16</f>
-        <v>1378636.30366815</v>
+        <v>1726373.73582105</v>
       </c>
       <c r="J18" s="15"/>
       <c r="K18" s="15"/>
@@ -10981,31 +11002,31 @@
       </c>
       <c r="C28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:C126)</f>
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="D28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:D126)</f>
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="E28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:E126)</f>
-        <v>2400000</v>
+        <v>2750000</v>
       </c>
       <c r="F28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:F126)</f>
-        <v>2400000</v>
+        <v>2750000</v>
       </c>
       <c r="G28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:G126)</f>
-        <v>3900000</v>
+        <v>4200000</v>
       </c>
       <c r="H28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:H126)</f>
-        <v>3900000</v>
+        <v>4200000</v>
       </c>
       <c r="I28" s="19" t="n">
         <f aca="false">SUM(Assumptions!$C$126:I126)</f>
-        <v>3900000</v>
+        <v>4200000</v>
       </c>
       <c r="L28" s="6" t="s">
         <v>113</v>
@@ -11024,27 +11045,27 @@
       </c>
       <c r="D29" s="19" t="n">
         <f aca="false">SUM('P&amp;L'!$C$75:D75)</f>
-        <v>-705396.151525491</v>
+        <v>-702396.151525491</v>
       </c>
       <c r="E29" s="19" t="n">
         <f aca="false">SUM('P&amp;L'!$C$75:E75)</f>
-        <v>-1445884.24976989</v>
+        <v>-1439794.24976989</v>
       </c>
       <c r="F29" s="19" t="n">
         <f aca="false">SUM('P&amp;L'!$C$75:F75)</f>
-        <v>-2332260.42219449</v>
+        <v>-2315487.72219449</v>
       </c>
       <c r="G29" s="19" t="n">
         <f aca="false">SUM('P&amp;L'!$C$75:G75)</f>
-        <v>-3251158.08225758</v>
+        <v>-3223382.20125759</v>
       </c>
       <c r="H29" s="19" t="n">
         <f aca="false">SUM('P&amp;L'!$C$75:H75)</f>
-        <v>-3923972.61636915</v>
+        <v>-3886363.45893915</v>
       </c>
       <c r="I29" s="19" t="n">
         <f aca="false">SUM('P&amp;L'!$C$75:I75)</f>
-        <v>-3710570.80037294</v>
+        <v>-3662833.36822004</v>
       </c>
       <c r="L29" s="6" t="s">
         <v>113</v>
@@ -11060,31 +11081,31 @@
       <c r="B30" s="15"/>
       <c r="C30" s="16" t="n">
         <f aca="false">C28 + C29</f>
-        <v>650195.079534884</v>
+        <v>750195.079534884</v>
       </c>
       <c r="D30" s="16" t="n">
         <f aca="false">D28 + D29</f>
-        <v>194603.848474509</v>
+        <v>297603.848474509</v>
       </c>
       <c r="E30" s="16" t="n">
         <f aca="false">E28 + E29</f>
-        <v>954115.750230114</v>
+        <v>1310205.75023011</v>
       </c>
       <c r="F30" s="16" t="n">
         <f aca="false">F28 + F29</f>
-        <v>67739.5778055103</v>
+        <v>434512.27780551</v>
       </c>
       <c r="G30" s="16" t="n">
         <f aca="false">G28 + G29</f>
-        <v>648841.917742415</v>
+        <v>976617.798742415</v>
       </c>
       <c r="H30" s="16" t="n">
         <f aca="false">H28 + H29</f>
-        <v>-23972.6163691478</v>
+        <v>313636.541060852</v>
       </c>
       <c r="I30" s="16" t="n">
         <f aca="false">I28 + I29</f>
-        <v>189429.199627058</v>
+        <v>537166.631779958</v>
       </c>
       <c r="J30" s="15"/>
       <c r="K30" s="15"/>
@@ -11117,31 +11138,31 @@
       <c r="B33" s="15"/>
       <c r="C33" s="16" t="n">
         <f aca="false">C25 + C30</f>
-        <v>656359.463096528</v>
+        <v>756359.463096528</v>
       </c>
       <c r="D33" s="16" t="n">
         <f aca="false">D25 + D30</f>
-        <v>222836.725186837</v>
+        <v>325836.725186837</v>
       </c>
       <c r="E33" s="16" t="n">
         <f aca="false">E25 + E30</f>
-        <v>1009373.28447669</v>
+        <v>1365463.28447669</v>
       </c>
       <c r="F33" s="16" t="n">
         <f aca="false">F25 + F30</f>
-        <v>184412.249038387</v>
+        <v>551184.949038387</v>
       </c>
       <c r="G33" s="16" t="n">
         <f aca="false">G25 + G30</f>
-        <v>913243.362947895</v>
+        <v>1241019.24394789</v>
       </c>
       <c r="H33" s="16" t="n">
         <f aca="false">H25 + H30</f>
-        <v>542261.267877428</v>
+        <v>879870.425307427</v>
       </c>
       <c r="I33" s="16" t="n">
         <f aca="false">I25 + I30</f>
-        <v>1378636.30366815</v>
+        <v>1726373.73582105</v>
       </c>
       <c r="J33" s="15"/>
       <c r="K33" s="15"/>
@@ -11243,11 +11264,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="50"/>
   </cols>
@@ -11316,7 +11337,7 @@
         <v>424</v>
       </c>
       <c r="B6" s="3" t="str">
-        <f aca="false">CHOOSE($B$5, "Base", "Downside", "Upside", "Reg Delay")</f>
+        <f aca="false">CHOOSE($B$5, "Base", "Downside", "Upside", "Reg Delay", "Best", "Worst")</f>
         <v>Base</v>
       </c>
     </row>
@@ -11353,13 +11374,19 @@
       <c r="E9" s="21" t="s">
         <v>430</v>
       </c>
+      <c r="F9" s="21" t="s">
+        <v>431</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>432</v>
+      </c>
       <c r="M9" s="20" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B10" s="43" t="n">
         <v>1</v>
@@ -11373,13 +11400,19 @@
       <c r="E10" s="43" t="n">
         <v>1</v>
       </c>
+      <c r="F10" s="43" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G10" s="43" t="n">
+        <v>0.8</v>
+      </c>
       <c r="M10" s="6" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B11" s="43" t="n">
         <v>1</v>
@@ -11393,13 +11426,19 @@
       <c r="E11" s="43" t="n">
         <v>1</v>
       </c>
+      <c r="F11" s="43" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G11" s="43" t="n">
+        <v>1.25</v>
+      </c>
       <c r="M11" s="6" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B12" s="43" t="n">
         <v>1</v>
@@ -11413,13 +11452,19 @@
       <c r="E12" s="43" t="n">
         <v>1</v>
       </c>
+      <c r="F12" s="43" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G12" s="43" t="n">
+        <v>1.5</v>
+      </c>
       <c r="M12" s="6" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B13" s="43" t="n">
         <v>1</v>
@@ -11433,13 +11478,19 @@
       <c r="E13" s="43" t="n">
         <v>1.05</v>
       </c>
+      <c r="F13" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="43" t="n">
+        <v>1.1</v>
+      </c>
       <c r="M13" s="6" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B14" s="43" t="n">
         <v>1</v>
@@ -11453,13 +11504,19 @@
       <c r="E14" s="43" t="n">
         <v>1</v>
       </c>
+      <c r="F14" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="43" t="n">
+        <v>1</v>
+      </c>
       <c r="M14" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B15" s="43" t="n">
         <v>1</v>
@@ -11473,13 +11530,19 @@
       <c r="E15" s="43" t="n">
         <v>1.4</v>
       </c>
+      <c r="F15" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="43" t="n">
+        <v>1.2</v>
+      </c>
       <c r="M15" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>0</v>
@@ -11493,363 +11556,439 @@
       <c r="E16" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M16" s="6" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>446</v>
-      </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
+        <v>447</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="B17" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="43" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G17" s="43" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
-        <v>447</v>
-      </c>
-      <c r="B18" s="44" t="n">
-        <f aca="false">CHOOSE($B$5, $B$10, $C$10, $D$10, $E$10)</f>
+      <c r="A18" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B18" s="43" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>448</v>
-      </c>
-      <c r="B19" s="44" t="n">
-        <f aca="false">CHOOSE($B$5, $B$11, $C$11, $D$11, $E$11)</f>
+      <c r="C18" s="43" t="n">
         <v>1</v>
       </c>
+      <c r="D18" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="43" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G18" s="43" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>451</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="B20" s="44" t="n">
-        <f aca="false">CHOOSE($B$5, $B$12, $C$12, $D$12, $E$12)</f>
+        <f aca="false">CHOOSE($B$5, $B$10, $C$10, $D$10, $E$10, $F$10, $G$10)</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B21" s="44" t="n">
-        <f aca="false">CHOOSE($B$5, $B$13, $C$13, $D$13, $E$13)</f>
+        <f aca="false">CHOOSE($B$5, $B$11, $C$11, $D$11, $E$11, $F$11, $G$11)</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B22" s="44" t="n">
-        <f aca="false">CHOOSE($B$5, $B$14, $C$14, $D$14, $E$14)</f>
+        <f aca="false">CHOOSE($B$5, $B$12, $C$12, $D$12, $E$12, $F$12, $G$12)</f>
         <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B23" s="44" t="n">
-        <f aca="false">CHOOSE($B$5, $B$15, $C$15, $D$15, $E$15)</f>
+        <f aca="false">CHOOSE($B$5, $B$13, $C$13, $D$13, $E$13, $F$13, $G$13)</f>
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>453</v>
-      </c>
-      <c r="B24" s="45" t="n">
-        <f aca="false">CHOOSE($B$5, $B$16, $C$16, $D$16, $E$16)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>454</v>
-      </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
+        <v>456</v>
+      </c>
+      <c r="B24" s="44" t="n">
+        <f aca="false">CHOOSE($B$5, $B$14, $C$14, $D$14, $E$14, $F$14, $G$14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>457</v>
+      </c>
+      <c r="B25" s="44" t="n">
+        <f aca="false">CHOOSE($B$5, $B$15, $C$15, $D$15, $E$15, $F$15, $G$15)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>458</v>
+      </c>
+      <c r="B26" s="45" t="n">
+        <f aca="false">CHOOSE($B$5, $B$16, $C$16, $D$16, $E$16, $F$16, $G$16)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
+        <v>459</v>
+      </c>
+      <c r="B27" s="44" t="n">
+        <f aca="false">CHOOSE($B$5, $B$17, $C$17, $D$17, $E$17, $F$17, $G$17)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
+        <v>460</v>
+      </c>
+      <c r="B28" s="44" t="n">
+        <f aca="false">CHOOSE($B$5, $B$18, $C$18, $D$18, $E$18, $F$18, $G$18)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="7"/>
+      <c r="K30" s="7"/>
+      <c r="L30" s="7"/>
+      <c r="M30" s="7"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
         <v>424</v>
       </c>
-      <c r="B27" s="46" t="str">
+      <c r="B31" s="46" t="str">
         <f aca="false">$B$6</f>
         <v>Base</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
-        <v>455</v>
-      </c>
-      <c r="B28" s="35" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>462</v>
+      </c>
+      <c r="B32" s="35" t="n">
         <f aca="false">'P&amp;L'!I14</f>
         <v>3978956.7</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
-        <v>456</v>
-      </c>
-      <c r="B29" s="35" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>463</v>
+      </c>
+      <c r="B33" s="35" t="n">
         <f aca="false">'P&amp;L'!I23</f>
         <v>2398120.695</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
-        <v>457</v>
-      </c>
-      <c r="B30" s="35" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>464</v>
+      </c>
+      <c r="B34" s="35" t="n">
         <f aca="false">'P&amp;L'!I58</f>
         <v>149150.695</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
-        <v>458</v>
-      </c>
-      <c r="B31" s="35" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
+        <v>465</v>
+      </c>
+      <c r="B35" s="35" t="n">
         <f aca="false">'P&amp;L'!I75</f>
-        <v>213401.815996206</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
-        <v>459</v>
-      </c>
-      <c r="B32" s="35" t="n">
+        <v>223530.090719106</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
+        <v>466</v>
+      </c>
+      <c r="B36" s="35" t="n">
         <f aca="false">'Cash flow'!I39</f>
-        <v>521193.539235669</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+        <v>868930.971388569</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
         <v>387</v>
       </c>
-      <c r="B33" s="35" t="n">
+      <c r="B37" s="35" t="n">
         <f aca="false">'Cash flow'!B47</f>
-        <v>-3746184.72869792</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
+        <v>-3708575.57126792</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
         <v>393</v>
       </c>
-      <c r="B34" s="46" t="str">
+      <c r="B38" s="46" t="str">
         <f aca="false">'Cash flow'!B52</f>
         <v>Y7</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
-        <v>460</v>
-      </c>
-      <c r="B35" s="35" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
+        <v>467</v>
+      </c>
+      <c r="B39" s="35" t="n">
         <f aca="false">'Cash flow'!B49</f>
-        <v>3900000</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
+        <v>4200000</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="7"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
         <v>426</v>
       </c>
-      <c r="B38" s="21" t="s">
-        <v>462</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>463</v>
-      </c>
-      <c r="D38" s="21" t="s">
-        <v>464</v>
-      </c>
-      <c r="M38" s="20" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="B39" s="19" t="n">
+      <c r="B42" s="21" t="s">
+        <v>469</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>471</v>
+      </c>
+      <c r="M42" s="20" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B43" s="19" t="n">
         <f aca="false">-0.2 * 'P&amp;L'!I23</f>
         <v>-479624.139</v>
       </c>
-      <c r="C39" s="19" t="n">
+      <c r="C43" s="19" t="n">
         <f aca="false">0.2 * 'P&amp;L'!I23</f>
         <v>479624.139</v>
       </c>
-      <c r="D39" s="19" t="n">
-        <f aca="false">MAX(ABS(B39), ABS(C39))</f>
+      <c r="D43" s="19" t="n">
+        <f aca="false">MAX(ABS(B43), ABS(C43))</f>
         <v>479624.139</v>
       </c>
-      <c r="M39" s="6" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="B40" s="19" t="n">
+      <c r="M43" s="6" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="B44" s="19" t="n">
         <f aca="false">-0.15 * 'P&amp;L'!I10 * 0.85</f>
         <v>-223368.10425</v>
       </c>
-      <c r="C40" s="19" t="n">
+      <c r="C44" s="19" t="n">
         <f aca="false">0.15 * 'P&amp;L'!I10 * 0.85</f>
         <v>223368.10425</v>
       </c>
-      <c r="D40" s="19" t="n">
-        <f aca="false">MAX(ABS(B40), ABS(C40))</f>
+      <c r="D44" s="19" t="n">
+        <f aca="false">MAX(ABS(B44), ABS(C44))</f>
         <v>223368.10425</v>
       </c>
-      <c r="M40" s="6" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
-        <v>470</v>
-      </c>
-      <c r="B41" s="19" t="n">
+      <c r="M44" s="6" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B45" s="19" t="n">
         <f aca="false">-0.3 * 'P&amp;L'!I17</f>
         <v>-395415</v>
       </c>
-      <c r="C41" s="19" t="n">
+      <c r="C45" s="19" t="n">
         <f aca="false">0.15 * 'P&amp;L'!I17</f>
         <v>197707.5</v>
       </c>
-      <c r="D41" s="19" t="n">
-        <f aca="false">MAX(ABS(B41), ABS(C41))</f>
+      <c r="D45" s="19" t="n">
+        <f aca="false">MAX(ABS(B45), ABS(C45))</f>
         <v>395415</v>
       </c>
-      <c r="M41" s="6" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
-        <v>472</v>
-      </c>
-      <c r="B42" s="19" t="n">
+      <c r="M45" s="6" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="B46" s="19" t="n">
         <f aca="false">-0.333 * 'P&amp;L'!I10 * 0.85</f>
         <v>-495877.191435</v>
       </c>
-      <c r="C42" s="19" t="n">
+      <c r="C46" s="19" t="n">
         <f aca="false">0.333 * 'P&amp;L'!I10 * 0.85</f>
         <v>495877.191435</v>
       </c>
-      <c r="D42" s="19" t="n">
-        <f aca="false">MAX(ABS(B42), ABS(C42))</f>
+      <c r="D46" s="19" t="n">
+        <f aca="false">MAX(ABS(B46), ABS(C46))</f>
         <v>495877.191435</v>
       </c>
-      <c r="M42" s="6" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="B43" s="19" t="n">
+      <c r="M46" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B47" s="19" t="n">
         <f aca="false">-0.15 * 'P&amp;L'!I9</f>
         <v>-334057.5</v>
       </c>
-      <c r="C43" s="19" t="n">
+      <c r="C47" s="19" t="n">
         <f aca="false">0.15 * 'P&amp;L'!I9</f>
         <v>334057.5</v>
       </c>
-      <c r="D43" s="19" t="n">
-        <f aca="false">MAX(ABS(B43), ABS(C43))</f>
+      <c r="D47" s="19" t="n">
+        <f aca="false">MAX(ABS(B47), ABS(C47))</f>
         <v>334057.5</v>
       </c>
-      <c r="M43" s="6" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
-        <v>476</v>
-      </c>
-      <c r="B44" s="19" t="n">
+      <c r="M47" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="B48" s="19" t="n">
         <f aca="false">-0.1 * Assumptions!I69</f>
         <v>-128897</v>
       </c>
-      <c r="C44" s="19" t="n">
+      <c r="C48" s="19" t="n">
         <f aca="false">0.1 * Assumptions!I69</f>
         <v>128897</v>
       </c>
-      <c r="D44" s="19" t="n">
-        <f aca="false">MAX(ABS(B44), ABS(C44))</f>
+      <c r="D48" s="19" t="n">
+        <f aca="false">MAX(ABS(B48), ABS(C48))</f>
         <v>128897</v>
       </c>
-      <c r="M44" s="6" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="20" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
+      <c r="M48" s="6" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="20" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
+      <c r="L51" s="2"/>
+      <c r="M51" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -11857,10 +11996,10 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="A8:M8"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="A26:M26"/>
-    <mergeCell ref="A37:M37"/>
-    <mergeCell ref="A47:M47"/>
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A51:M51"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>